<commit_message>
Add Day 2: writing, reading and extraction, data, presentations
- slides/day2.html: 50 slides over four sessions (Arabic correspondence and translation with a
  glossary; summaries, extraction with evidence, transcript to minutes, like-for-like quote
  comparison; computing with code, text classification, broken formulas; decision stories,
  conclusion titles, RICE for images, disclosure)
- labs D2_1 to D2_4 with instructor keys
- File pack: training budget now reconciles with the quarterly report (484,100 planned,
  370,000 spent); the report summary no longer miscounts KPIs below target
</commit_message>
<xml_diff>
--- a/labs/files/training_budget_2026.xlsx
+++ b/labs/files/training_budget_2026.xlsx
@@ -567,25 +567,25 @@
         <v>9</v>
       </c>
       <c r="C2" s="3">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D2" s="3">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="E2" s="3">
         <f>C2*D2</f>
-        <v>60000</v>
+        <v>36000</v>
       </c>
       <c r="F2" s="3">
-        <v>52000</v>
+        <v>36000</v>
       </c>
       <c r="G2" s="3">
         <f>E2-F2</f>
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="H2" s="4">
         <f>F2/E2</f>
-        <v>0.8666666666666667</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -599,18 +599,18 @@
         <v>40</v>
       </c>
       <c r="D3" s="3">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="E3" s="3">
         <f>C3*D3</f>
-        <v>36000</v>
+        <v>24000</v>
       </c>
       <c r="F3" s="3">
         <v>0</v>
       </c>
       <c r="G3" s="3">
         <f>E3-F3</f>
-        <v>36000</v>
+        <v>24000</v>
       </c>
       <c r="H3" s="4">
         <f>F3/E3</f>
@@ -625,25 +625,25 @@
         <v>12</v>
       </c>
       <c r="C4" s="3">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="D4" s="3">
-        <v>2200</v>
+        <v>1500</v>
       </c>
       <c r="E4" s="3">
         <f>C4*D4</f>
-        <v>132000</v>
+        <v>60000</v>
       </c>
       <c r="F4" s="3">
-        <v>61000</v>
+        <v>45000</v>
       </c>
       <c r="G4" s="3">
         <f>E4-F4</f>
-        <v>71000</v>
+        <v>15000</v>
       </c>
       <c r="H4" s="4">
         <f>F4/E4</f>
-        <v>0.4621212121212121</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -682,25 +682,25 @@
         <v>16</v>
       </c>
       <c r="C6" s="3">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D6" s="3">
         <v>4200</v>
       </c>
       <c r="E6" s="3">
         <f>C6*D6</f>
-        <v>50400</v>
+        <v>33600</v>
       </c>
       <c r="F6" s="3">
-        <v>30400</v>
+        <v>25200</v>
       </c>
       <c r="G6" s="3">
         <f>E6-F6</f>
-        <v>20000</v>
+        <v>8400</v>
       </c>
       <c r="H6" s="4">
         <f>F6/E6</f>
-        <v>0.6031746031746031</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -743,22 +743,22 @@
         <v>45</v>
       </c>
       <c r="D8" s="3">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="E8" s="3">
         <f>C8*D8</f>
-        <v>36000</v>
+        <v>27000</v>
       </c>
       <c r="F8" s="3">
         <v>21600</v>
       </c>
       <c r="G8" s="3">
         <f>E8-F8</f>
-        <v>14400</v>
+        <v>5400</v>
       </c>
       <c r="H8" s="4">
         <f>F8/E8</f>
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -772,18 +772,18 @@
         <v>120</v>
       </c>
       <c r="D9" s="3">
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="E9" s="3">
         <f>C9*D9</f>
-        <v>42000</v>
+        <v>30000</v>
       </c>
       <c r="F9" s="3">
-        <v>42000</v>
+        <v>30000</v>
       </c>
       <c r="G9" s="3">
         <f>E9-F8</f>
-        <v>20400</v>
+        <v>8400</v>
       </c>
       <c r="H9" s="4">
         <f>F9/E9</f>
@@ -798,25 +798,25 @@
         <v>22</v>
       </c>
       <c r="C10" s="3">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D10" s="3">
         <v>6500</v>
       </c>
       <c r="E10" s="3">
         <f>C10*D10</f>
-        <v>91000</v>
+        <v>52000</v>
       </c>
       <c r="F10" s="3">
-        <v>52000</v>
+        <v>41600</v>
       </c>
       <c r="G10" s="3">
         <f>E10-F10</f>
-        <v>39000</v>
+        <v>10400</v>
       </c>
       <c r="H10" s="4">
         <f>F10/E10</f>
-        <v>0.5714285714285714</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -827,25 +827,25 @@
         <v>24</v>
       </c>
       <c r="C11" s="3">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D11" s="3">
         <v>2400</v>
       </c>
       <c r="E11" s="3">
         <f>C11*D11</f>
-        <v>43200</v>
+        <v>28800</v>
       </c>
       <c r="F11" s="3">
         <v>19200</v>
       </c>
       <c r="G11" s="3">
         <f>E11-F11</f>
-        <v>24000</v>
+        <v>9600</v>
       </c>
       <c r="H11" s="4">
         <f>F11/E11</f>
-        <v>0.4444444444444444</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -885,21 +885,21 @@
         <v>18</v>
       </c>
       <c r="C13" s="3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D13" s="3">
         <v>14500</v>
       </c>
       <c r="E13" s="3">
         <f>C13*D13</f>
-        <v>116000</v>
+        <v>58000</v>
       </c>
       <c r="F13" s="3">
-        <v>58000</v>
+        <v>29000</v>
       </c>
       <c r="G13" s="3">
         <f>E13-F13</f>
-        <v>58000</v>
+        <v>29000</v>
       </c>
       <c r="H13" s="4">
         <f>F13/E13</f>
@@ -953,15 +953,15 @@
         <v>19000</v>
       </c>
       <c r="F15" s="3">
-        <v>15200</v>
+        <v>19000</v>
       </c>
       <c r="G15" s="3">
         <f>E15-F15</f>
-        <v>3800</v>
+        <v>0</v>
       </c>
       <c r="H15" s="4">
         <f>F15/E15</f>
-        <v>0.8</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -971,7 +971,7 @@
       <c r="B16" s="5"/>
       <c r="C16" s="5">
         <f>SUM(C2:C15)</f>
-        <v>422</v>
+        <v>372</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5" t="e">
@@ -980,7 +980,7 @@
       </c>
       <c r="F16" s="5">
         <f>SUM(F2:F15)</f>
-        <v>454800</v>
+        <v>370000</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>

</xml_diff>